<commit_message>
Services engagements below target; under budget flagged like over; Export menu without Copy a link
- Three September services engagements below the 40% target (reasons in financial_model.py); all CSVs, schema,
  table guide, Power BI prompts and downloads rebuilt from the model.
- Grant budget chart: off budget either way is red, within 1% amber (site, PDF, PowerPoint).
- Export menu: Copy a link row removed sitewide, menu narrower; the hero's menu opens upwards and nothing clips it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/media/exports/reports/2026-08/growth.xlsx
+++ b/media/exports/reports/2026-08/growth.xlsx
@@ -1047,7 +1047,7 @@
     <row r="70" ht="60" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>August's client work made $68,860 gross margin (60.1%). Consultant time not charged to client work took $7,620 and overheads $53,650, leaving $7,590 profit before tax (6.6% of revenue). To cover overheads, client work needs a 53.4% gross margin on average. (Workings sheet: "From gross margin to profit".)</t>
+          <t>August's client work made $68,020 gross margin (59.3%). Consultant time not charged to client work took $6,780 and overheads $53,650, leaving $7,590 profit before tax (6.6% of revenue). To cover overheads, client work needs a 52.7% gross margin on average. (Workings sheet: "From gross margin to profit".)</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>$141,935 before overheads</t>
+          <t>$141,095 before overheads</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1135,7 @@
     <row r="79" ht="45" customHeight="1">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Revenue is 59.3% up on the same period last year, year to date ($235,395 against $147,795). Training makes the highest gross margin (68.4%); Projects the lowest (58.9%). The business needs 53.4% gross margin just to cover overheads.</t>
+          <t>Revenue is 59.3% up on the same period last year, year to date ($235,395 against $147,795). Training makes the highest gross margin (68.4%); Projects the lowest (58.9%). The business needs 52.7% gross margin just to cover overheads.</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>Training: 68.4% gross margin, the most profitable work you do. Projects: 58.9% gross margin, the thinnest, still above the 53.4% overheads need.</t>
+          <t>Training: 68.4% gross margin, the most profitable work you do. Projects: 58.9% gross margin, the thinnest, still above the 52.7% overheads need.</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>Projects brought in $155,195 this financial year to date, 49.8% on the same period last year (slower than the business as a whole, 59.3%), at a 58.9% gross margin (below the 60.3% overall).</t>
+          <t>Projects brought in $155,195 this financial year to date, 49.8% on the same period last year (slower than the business as a whole, 59.3%), at a 58.9% gross margin (below the 59.9% overall).</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1253,7 @@
     <row r="94" ht="30" customHeight="1">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>Projects: 58.9% gross margin, 5.5 points clear of the 53.4% overheads need.</t>
+          <t>Projects: 58.9% gross margin, 6.2 points clear of the 52.7% overheads need.</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="C100" s="10" t="inlineStr">
         <is>
-          <t>$40,100 before overheads</t>
+          <t>$39,260 before overheads</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
     <row r="103" ht="30" customHeight="1">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>Retainers brought in $65,000 this financial year to date, 99.4% on the same period last year (faster than the business as a whole, 59.3%), at a 61.7% gross margin (above the 60.3% overall).</t>
+          <t>Retainers brought in $65,000 this financial year to date, 99.4% on the same period last year (faster than the business as a whole, 59.3%), at a 60.4% gross margin (above the 59.9% overall).</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1356,7 @@
     <row r="106" ht="30" customHeight="1">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>Retainers: 61.7% gross margin, 8.2 points clear of the 53.4% overheads need.</t>
+          <t>Retainers: 60.4% gross margin, 7.7 points clear of the 52.7% overheads need.</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1444,7 @@
     <row r="115" ht="30" customHeight="1">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Training brought in $15,200 this financial year to date, 31.0% on the same period last year (slower than the business as a whole, 59.3%), at a 68.4% gross margin (above the 60.3% overall).</t>
+          <t>Training brought in $15,200 this financial year to date, 31.0% on the same period last year (slower than the business as a whole, 59.3%), at a 68.4% gross margin (above the 59.9% overall).</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1459,7 @@
     <row r="118" ht="30" customHeight="1">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>Training: 68.4% gross margin, 15.0 points clear of the 53.4% overheads need.</t>
+          <t>Training: 68.4% gross margin, 15.7 points clear of the 52.7% overheads need.</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2566,7 @@
         </is>
       </c>
       <c r="B137" s="12" t="n">
-        <v>68860</v>
+        <v>68020</v>
       </c>
     </row>
     <row r="138">
@@ -2586,7 +2586,7 @@
         </is>
       </c>
       <c r="B139" s="12" t="n">
-        <v>38880</v>
+        <v>39720</v>
       </c>
     </row>
     <row r="140">
@@ -2799,7 +2799,7 @@
         </is>
       </c>
       <c r="B165" s="12" t="n">
-        <v>141935</v>
+        <v>141095</v>
       </c>
     </row>
     <row r="166">
@@ -2875,7 +2875,7 @@
         </is>
       </c>
       <c r="B175" s="12" t="n">
-        <v>141935</v>
+        <v>141095</v>
       </c>
     </row>
     <row r="176">
@@ -3213,7 +3213,7 @@
         </is>
       </c>
       <c r="B221" s="12" t="n">
-        <v>40100</v>
+        <v>39260</v>
       </c>
     </row>
     <row r="222">
@@ -3289,7 +3289,7 @@
         </is>
       </c>
       <c r="B231" s="12" t="n">
-        <v>40100</v>
+        <v>39260</v>
       </c>
     </row>
     <row r="232">
@@ -7449,7 +7449,7 @@
         <v>114640</v>
       </c>
       <c r="E28" s="12" t="n">
-        <v>45780</v>
+        <v>46620</v>
       </c>
       <c r="F28" s="12">
         <f>D28-E28</f>
@@ -8875,7 +8875,7 @@
         <v>32500</v>
       </c>
       <c r="E74" s="12" t="n">
-        <v>12000</v>
+        <v>12840</v>
       </c>
       <c r="F74" s="12">
         <f>D74-E74</f>
@@ -9731,7 +9731,7 @@
         <v/>
       </c>
       <c r="E7" s="12" t="n">
-        <v>40100</v>
+        <v>39260</v>
       </c>
       <c r="F7" s="13">
         <f>IF(B7=0,"",E7/B7)</f>
@@ -9779,7 +9779,7 @@
         <v/>
       </c>
       <c r="E9" s="12" t="n">
-        <v>141935</v>
+        <v>141095</v>
       </c>
       <c r="F9" s="13">
         <f>IF(B9=0,"",E9/B9)</f>

</xml_diff>